<commit_message>
fix(bd): agregar scope de carrera a prerrequisitos (bug MAT030)
prerrequisito era una tabla global sin distinguir carrera. Un curso
compartido (MAT002) con requisitos distintos segun la hoja del Excel
(TOPO: MAT001, ISI: MAT030) causaba que el loader insertara la union
de ambos, rompiendo el flujo de TOPO.

- Agrega columna id_carrera nullable a prerrequisito (NULL = aplica a
  todas las carreras que comparten el curso, valor = solo esa carrera)
- Actualiza el motor de prerrequisitos y el filtro de ofertas por
  banner_program scoped a carrera
- Corrige FIY423->MAT002 en el Excel (prerrequisito invalido, mismo
  ciclo)
- Corrige etiqueta de Estudios Generales para codigos reales de
  Banner (EGA/EGC/EGF/EGS)
- Elimina 17 secciones huerfanas en BD
- Consolida migraciones V1-V8 en V1__schema_inicial.sql

45/45 tests de integracion pasando, tsc limpio, verificado con curl
contra BD real.
</commit_message>
<xml_diff>
--- a/data-extractor/input/PLANES_DE_ESTUDIO.xlsx
+++ b/data-extractor/input/PLANES_DE_ESTUDIO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jafet\Documents\Personal\Sistema_Cursos\Sistema-Horarios\data-extractor\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C1B31CC-060E-48D3-B175-ECD20F2D2ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6750417F-3900-45E0-A2ED-7FA27978C758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LEEME" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1810" uniqueCount="570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1810" uniqueCount="572">
   <si>
     <t>Ingeniería en Sistemas de Información — Bachillerato</t>
   </si>
@@ -861,9 +861,6 @@
     <t>Física I para Topografía</t>
   </si>
   <si>
-    <t>MAT001, MAT002</t>
-  </si>
-  <si>
     <t>FIY423L</t>
   </si>
   <si>
@@ -1735,6 +1732,15 @@
   </si>
   <si>
     <t xml:space="preserve">   no transcritas aquí — el alcance actual de SIHA cubre bachillerato; se pueden agregar después si aplica.</t>
+  </si>
+  <si>
+    <t>FIY423L, MAT002</t>
+  </si>
+  <si>
+    <t>FIY423, MAT002</t>
+  </si>
+  <si>
+    <t>FIY423L, FIY423</t>
   </si>
 </sst>
 </file>
@@ -5256,7 +5262,7 @@
       <c r="B11" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="13" t="s">
         <v>276</v>
       </c>
       <c r="D11" s="8" t="s">
@@ -5265,14 +5271,14 @@
       <c r="E11" s="7">
         <v>3</v>
       </c>
-      <c r="F11" s="8" t="s">
-        <v>278</v>
-      </c>
-      <c r="G11" s="8" t="s">
+      <c r="F11" s="11" t="s">
+        <v>269</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>569</v>
+      </c>
+      <c r="H11" s="8" t="s">
         <v>279</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="79.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -5282,23 +5288,23 @@
       <c r="B12" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>279</v>
+      <c r="C12" s="13" t="s">
+        <v>278</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E12" s="7">
         <v>1</v>
       </c>
-      <c r="F12" s="8" t="s">
-        <v>278</v>
-      </c>
-      <c r="G12" s="8" t="s">
-        <v>276</v>
+      <c r="F12" s="11" t="s">
+        <v>269</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>570</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -5320,8 +5326,8 @@
       <c r="F13" s="8" t="s">
         <v>269</v>
       </c>
-      <c r="G13" s="8" t="s">
-        <v>13</v>
+      <c r="G13" s="11" t="s">
+        <v>571</v>
       </c>
       <c r="H13" s="8" t="s">
         <v>270</v>
@@ -5335,10 +5341,10 @@
         <v>21</v>
       </c>
       <c r="C14" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="D14" s="8" t="s">
         <v>282</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>283</v>
       </c>
       <c r="E14" s="7">
         <v>3</v>
@@ -5413,16 +5419,16 @@
         <v>10</v>
       </c>
       <c r="C17" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>284</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="E17" s="7">
+        <v>3</v>
+      </c>
+      <c r="F17" s="8" t="s">
         <v>285</v>
-      </c>
-      <c r="E17" s="7">
-        <v>3</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>286</v>
       </c>
       <c r="G17" s="8" t="s">
         <v>13</v>
@@ -5439,22 +5445,22 @@
         <v>10</v>
       </c>
       <c r="C18" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="D18" s="8" t="s">
         <v>287</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="E18" s="7">
+        <v>3</v>
+      </c>
+      <c r="F18" s="8" t="s">
         <v>288</v>
       </c>
-      <c r="E18" s="7">
-        <v>3</v>
-      </c>
-      <c r="F18" s="8" t="s">
+      <c r="G18" s="8" t="s">
         <v>289</v>
       </c>
-      <c r="G18" s="8" t="s">
-        <v>290</v>
-      </c>
       <c r="H18" s="8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="79.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -5465,22 +5471,22 @@
         <v>10</v>
       </c>
       <c r="C19" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="D19" s="8" t="s">
         <v>290</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>291</v>
       </c>
       <c r="E19" s="7">
         <v>1</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -5491,10 +5497,10 @@
         <v>10</v>
       </c>
       <c r="C20" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="D20" s="8" t="s">
         <v>292</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>293</v>
       </c>
       <c r="E20" s="7">
         <v>4</v>
@@ -5517,16 +5523,16 @@
         <v>10</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E21" s="7">
         <v>3</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="G21" s="8" t="s">
         <v>13</v>
@@ -5546,7 +5552,7 @@
         <v>19</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E22" s="7">
         <v>4</v>
@@ -5569,16 +5575,16 @@
         <v>21</v>
       </c>
       <c r="C23" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="D23" s="8" t="s">
         <v>296</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>297</v>
       </c>
       <c r="E23" s="7">
         <v>2</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G23" s="8" t="s">
         <v>13</v>
@@ -5595,16 +5601,16 @@
         <v>21</v>
       </c>
       <c r="C24" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="D24" s="8" t="s">
         <v>299</v>
-      </c>
-      <c r="D24" s="8" t="s">
-        <v>300</v>
       </c>
       <c r="E24" s="7">
         <v>2</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G24" s="8" t="s">
         <v>13</v>
@@ -5621,16 +5627,16 @@
         <v>21</v>
       </c>
       <c r="C25" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="D25" s="8" t="s">
         <v>301</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="E25" s="7">
+        <v>3</v>
+      </c>
+      <c r="F25" s="8" t="s">
         <v>302</v>
-      </c>
-      <c r="E25" s="7">
-        <v>3</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>303</v>
       </c>
       <c r="G25" s="8" t="s">
         <v>13</v>
@@ -5650,7 +5656,7 @@
         <v>33</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E26" s="7">
         <v>4</v>
@@ -5676,7 +5682,7 @@
         <v>52</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E27" s="7">
         <v>3</v>
@@ -5702,7 +5708,7 @@
         <v>29</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="E28" s="7">
         <v>4</v>
@@ -5725,16 +5731,16 @@
         <v>10</v>
       </c>
       <c r="C29" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="D29" s="8" t="s">
         <v>307</v>
       </c>
-      <c r="D29" s="8" t="s">
-        <v>308</v>
-      </c>
       <c r="E29" s="7">
         <v>3</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G29" s="8" t="s">
         <v>13</v>
@@ -5751,16 +5757,16 @@
         <v>10</v>
       </c>
       <c r="C30" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="D30" s="8" t="s">
         <v>309</v>
       </c>
-      <c r="D30" s="8" t="s">
-        <v>310</v>
-      </c>
       <c r="E30" s="7">
         <v>3</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G30" s="8" t="s">
         <v>13</v>
@@ -5777,16 +5783,16 @@
         <v>10</v>
       </c>
       <c r="C31" s="7" t="s">
+        <v>310</v>
+      </c>
+      <c r="D31" s="8" t="s">
         <v>311</v>
       </c>
-      <c r="D31" s="8" t="s">
-        <v>312</v>
-      </c>
       <c r="E31" s="7">
         <v>3</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G31" s="8" t="s">
         <v>13</v>
@@ -5803,16 +5809,16 @@
         <v>10</v>
       </c>
       <c r="C32" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="D32" s="8" t="s">
         <v>313</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>314</v>
       </c>
       <c r="E32" s="7">
         <v>4</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="G32" s="8" t="s">
         <v>13</v>
@@ -5829,10 +5835,10 @@
         <v>10</v>
       </c>
       <c r="C33" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="D33" s="8" t="s">
         <v>315</v>
-      </c>
-      <c r="D33" s="8" t="s">
-        <v>316</v>
       </c>
       <c r="E33" s="7">
         <v>2</v>
@@ -5858,7 +5864,7 @@
         <v>179</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E34" s="7">
         <v>3</v>
@@ -5881,16 +5887,16 @@
         <v>21</v>
       </c>
       <c r="C35" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="D35" s="8" t="s">
         <v>318</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>319</v>
       </c>
       <c r="E35" s="7">
         <v>4</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="G35" s="8" t="s">
         <v>13</v>
@@ -5907,16 +5913,16 @@
         <v>21</v>
       </c>
       <c r="C36" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="D36" s="8" t="s">
         <v>321</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>322</v>
       </c>
       <c r="E36" s="7">
         <v>4</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G36" s="8" t="s">
         <v>13</v>
@@ -5933,16 +5939,16 @@
         <v>21</v>
       </c>
       <c r="C37" s="7" t="s">
+        <v>322</v>
+      </c>
+      <c r="D37" s="8" t="s">
         <v>323</v>
       </c>
-      <c r="D37" s="8" t="s">
+      <c r="E37" s="7">
+        <v>3</v>
+      </c>
+      <c r="F37" s="8" t="s">
         <v>324</v>
-      </c>
-      <c r="E37" s="7">
-        <v>3</v>
-      </c>
-      <c r="F37" s="8" t="s">
-        <v>325</v>
       </c>
       <c r="G37" s="8" t="s">
         <v>13</v>
@@ -5959,16 +5965,16 @@
         <v>21</v>
       </c>
       <c r="C38" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="D38" s="8" t="s">
         <v>326</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>327</v>
       </c>
       <c r="E38" s="7">
         <v>4</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="G38" s="8" t="s">
         <v>13</v>
@@ -5988,7 +5994,7 @@
         <v>179</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="E39" s="7">
         <v>3</v>
@@ -6011,16 +6017,16 @@
         <v>10</v>
       </c>
       <c r="C40" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="D40" s="8" t="s">
         <v>329</v>
       </c>
-      <c r="D40" s="8" t="s">
-        <v>330</v>
-      </c>
       <c r="E40" s="7">
         <v>3</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="G40" s="8" t="s">
         <v>13</v>
@@ -6037,16 +6043,16 @@
         <v>10</v>
       </c>
       <c r="C41" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="D41" s="8" t="s">
         <v>331</v>
       </c>
-      <c r="D41" s="8" t="s">
-        <v>332</v>
-      </c>
       <c r="E41" s="7">
         <v>3</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G41" s="8" t="s">
         <v>13</v>
@@ -6063,16 +6069,16 @@
         <v>10</v>
       </c>
       <c r="C42" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="D42" s="8" t="s">
         <v>333</v>
       </c>
-      <c r="D42" s="8" t="s">
-        <v>334</v>
-      </c>
       <c r="E42" s="7">
         <v>3</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="G42" s="8" t="s">
         <v>13</v>
@@ -6089,16 +6095,16 @@
         <v>10</v>
       </c>
       <c r="C43" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="D43" s="8" t="s">
         <v>335</v>
       </c>
-      <c r="D43" s="8" t="s">
-        <v>336</v>
-      </c>
       <c r="E43" s="7">
         <v>3</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G43" s="8" t="s">
         <v>13</v>
@@ -6115,16 +6121,16 @@
         <v>10</v>
       </c>
       <c r="C44" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="D44" s="8" t="s">
         <v>337</v>
       </c>
-      <c r="D44" s="8" t="s">
-        <v>338</v>
-      </c>
       <c r="E44" s="7">
         <v>3</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="G44" s="8" t="s">
         <v>13</v>
@@ -6144,7 +6150,7 @@
         <v>179</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E45" s="7">
         <v>3</v>
@@ -6167,16 +6173,16 @@
         <v>21</v>
       </c>
       <c r="C46" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="D46" s="8" t="s">
         <v>340</v>
       </c>
-      <c r="D46" s="8" t="s">
-        <v>341</v>
-      </c>
       <c r="E46" s="7">
         <v>3</v>
       </c>
       <c r="F46" s="8" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="G46" s="8" t="s">
         <v>13</v>
@@ -6193,16 +6199,16 @@
         <v>21</v>
       </c>
       <c r="C47" s="7" t="s">
+        <v>341</v>
+      </c>
+      <c r="D47" s="8" t="s">
         <v>342</v>
       </c>
-      <c r="D47" s="8" t="s">
-        <v>343</v>
-      </c>
       <c r="E47" s="7">
         <v>3</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="G47" s="8" t="s">
         <v>13</v>
@@ -6219,22 +6225,22 @@
         <v>21</v>
       </c>
       <c r="C48" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="D48" s="8" t="s">
         <v>344</v>
-      </c>
-      <c r="D48" s="8" t="s">
-        <v>345</v>
       </c>
       <c r="E48" s="7">
         <v>4</v>
       </c>
       <c r="F48" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="G48" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H48" s="8" t="s">
         <v>346</v>
-      </c>
-      <c r="G48" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H48" s="8" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="66" customHeight="1" x14ac:dyDescent="0.3">
@@ -6245,22 +6251,22 @@
         <v>21</v>
       </c>
       <c r="C49" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="D49" s="8" t="s">
         <v>348</v>
-      </c>
-      <c r="D49" s="8" t="s">
-        <v>349</v>
       </c>
       <c r="E49" s="7">
         <v>4</v>
       </c>
       <c r="F49" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="G49" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H49" s="8" t="s">
         <v>346</v>
-      </c>
-      <c r="G49" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H49" s="8" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6274,7 +6280,7 @@
         <v>179</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E50" s="7">
         <v>3</v>
@@ -6297,22 +6303,22 @@
         <v>13</v>
       </c>
       <c r="C51" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="D51" s="8" t="s">
         <v>351</v>
       </c>
-      <c r="D51" s="8" t="s">
+      <c r="E51" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F51" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="G51" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H51" s="8" t="s">
         <v>352</v>
-      </c>
-      <c r="E51" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F51" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G51" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H51" s="8" t="s">
-        <v>353</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
@@ -6323,22 +6329,22 @@
         <v>13</v>
       </c>
       <c r="C52" s="7" t="s">
+        <v>353</v>
+      </c>
+      <c r="D52" s="8" t="s">
         <v>354</v>
       </c>
-      <c r="D52" s="8" t="s">
+      <c r="E52" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F52" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="G52" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H52" s="8" t="s">
         <v>355</v>
-      </c>
-      <c r="E52" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F52" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G52" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H52" s="8" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.3">
@@ -6349,11 +6355,11 @@
         <v>13</v>
       </c>
       <c r="C53" s="7" t="s">
+        <v>356</v>
+      </c>
+      <c r="D53" s="8" t="s">
         <v>357</v>
       </c>
-      <c r="D53" s="8" t="s">
-        <v>358</v>
-      </c>
       <c r="E53" s="7" t="s">
         <v>13</v>
       </c>
@@ -6364,7 +6370,7 @@
         <v>13</v>
       </c>
       <c r="H53" s="8" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.3">
@@ -6375,11 +6381,11 @@
         <v>13</v>
       </c>
       <c r="C54" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="D54" s="8" t="s">
         <v>359</v>
       </c>
-      <c r="D54" s="8" t="s">
-        <v>360</v>
-      </c>
       <c r="E54" s="7" t="s">
         <v>13</v>
       </c>
@@ -6390,7 +6396,7 @@
         <v>13</v>
       </c>
       <c r="H54" s="8" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.3">
@@ -6401,11 +6407,11 @@
         <v>13</v>
       </c>
       <c r="C55" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="D55" s="8" t="s">
         <v>361</v>
       </c>
-      <c r="D55" s="8" t="s">
-        <v>362</v>
-      </c>
       <c r="E55" s="7" t="s">
         <v>13</v>
       </c>
@@ -6416,7 +6422,7 @@
         <v>13</v>
       </c>
       <c r="H55" s="8" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="56" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6427,10 +6433,10 @@
         <v>13</v>
       </c>
       <c r="C56" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="D56" s="8" t="s">
         <v>363</v>
-      </c>
-      <c r="D56" s="8" t="s">
-        <v>364</v>
       </c>
       <c r="E56" s="7">
         <v>4</v>
@@ -6442,7 +6448,7 @@
         <v>13</v>
       </c>
       <c r="H56" s="8" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.3">
@@ -6453,11 +6459,11 @@
         <v>13</v>
       </c>
       <c r="C57" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="D57" s="8" t="s">
         <v>365</v>
       </c>
-      <c r="D57" s="8" t="s">
-        <v>366</v>
-      </c>
       <c r="E57" s="7" t="s">
         <v>13</v>
       </c>
@@ -6468,57 +6474,57 @@
         <v>13</v>
       </c>
       <c r="H57" s="8" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" s="9" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" s="9" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" s="9" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" s="9" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" s="9" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" s="9" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65" s="9" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A66" s="9" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A67" s="9" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A68" s="9" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
   </sheetData>
@@ -6542,12 +6548,12 @@
   <sheetData>
     <row r="1" spans="1:8" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -6599,7 +6605,7 @@
         <v>13</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6625,7 +6631,7 @@
         <v>13</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6651,7 +6657,7 @@
         <v>13</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6662,10 +6668,10 @@
         <v>10</v>
       </c>
       <c r="C8" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>380</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>381</v>
       </c>
       <c r="E8" s="7">
         <v>4</v>
@@ -6677,7 +6683,7 @@
         <v>13</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6691,7 +6697,7 @@
         <v>19</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E9" s="7">
         <v>4</v>
@@ -6703,7 +6709,7 @@
         <v>13</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6729,7 +6735,7 @@
         <v>13</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6755,7 +6761,7 @@
         <v>13</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6781,7 +6787,7 @@
         <v>13</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6795,7 +6801,7 @@
         <v>29</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E13" s="7">
         <v>4</v>
@@ -6807,7 +6813,7 @@
         <v>13</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6818,22 +6824,22 @@
         <v>21</v>
       </c>
       <c r="C14" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="D14" s="8" t="s">
         <v>384</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>385</v>
       </c>
       <c r="E14" s="7">
         <v>4</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="G14" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6847,7 +6853,7 @@
         <v>33</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E15" s="7">
         <v>4</v>
@@ -6859,7 +6865,7 @@
         <v>13</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6870,22 +6876,22 @@
         <v>10</v>
       </c>
       <c r="C16" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>386</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>387</v>
       </c>
       <c r="E16" s="7">
         <v>4</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="G16" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6896,10 +6902,10 @@
         <v>10</v>
       </c>
       <c r="C17" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>388</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>389</v>
       </c>
       <c r="E17" s="7">
         <v>3</v>
@@ -6911,7 +6917,7 @@
         <v>13</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6922,22 +6928,22 @@
         <v>10</v>
       </c>
       <c r="C18" s="7" t="s">
+        <v>389</v>
+      </c>
+      <c r="D18" s="8" t="s">
         <v>390</v>
       </c>
-      <c r="D18" s="8" t="s">
-        <v>391</v>
-      </c>
       <c r="E18" s="7">
         <v>3</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="G18" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6948,22 +6954,22 @@
         <v>10</v>
       </c>
       <c r="C19" s="7" t="s">
+        <v>391</v>
+      </c>
+      <c r="D19" s="8" t="s">
         <v>392</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>393</v>
       </c>
       <c r="E19" s="7">
         <v>4</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="G19" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -6974,22 +6980,22 @@
         <v>21</v>
       </c>
       <c r="C20" s="7" t="s">
+        <v>393</v>
+      </c>
+      <c r="D20" s="8" t="s">
         <v>394</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>395</v>
       </c>
       <c r="E20" s="7">
         <v>4</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="G20" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7000,22 +7006,22 @@
         <v>21</v>
       </c>
       <c r="C21" s="7" t="s">
+        <v>395</v>
+      </c>
+      <c r="D21" s="8" t="s">
         <v>396</v>
       </c>
-      <c r="D21" s="8" t="s">
-        <v>397</v>
-      </c>
       <c r="E21" s="7">
         <v>3</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="G21" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7026,22 +7032,22 @@
         <v>21</v>
       </c>
       <c r="C22" s="7" t="s">
+        <v>397</v>
+      </c>
+      <c r="D22" s="8" t="s">
         <v>398</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="E22" s="7">
+        <v>3</v>
+      </c>
+      <c r="F22" s="8" t="s">
         <v>399</v>
       </c>
-      <c r="E22" s="7">
-        <v>3</v>
-      </c>
-      <c r="F22" s="8" t="s">
-        <v>400</v>
-      </c>
       <c r="G22" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7052,22 +7058,22 @@
         <v>21</v>
       </c>
       <c r="C23" s="7" t="s">
+        <v>400</v>
+      </c>
+      <c r="D23" s="8" t="s">
         <v>401</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>402</v>
       </c>
       <c r="E23" s="7">
         <v>4</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="G23" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7078,22 +7084,22 @@
         <v>21</v>
       </c>
       <c r="C24" s="7" t="s">
+        <v>402</v>
+      </c>
+      <c r="D24" s="8" t="s">
         <v>403</v>
-      </c>
-      <c r="D24" s="8" t="s">
-        <v>404</v>
       </c>
       <c r="E24" s="7">
         <v>4</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="G24" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7104,22 +7110,22 @@
         <v>10</v>
       </c>
       <c r="C25" s="7" t="s">
+        <v>404</v>
+      </c>
+      <c r="D25" s="8" t="s">
         <v>405</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>406</v>
       </c>
       <c r="E25" s="7">
         <v>4</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="G25" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7130,22 +7136,22 @@
         <v>10</v>
       </c>
       <c r="C26" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="D26" s="8" t="s">
         <v>408</v>
       </c>
-      <c r="D26" s="8" t="s">
-        <v>409</v>
-      </c>
       <c r="E26" s="7">
         <v>3</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G26" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7156,22 +7162,22 @@
         <v>10</v>
       </c>
       <c r="C27" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="D27" s="8" t="s">
         <v>410</v>
-      </c>
-      <c r="D27" s="8" t="s">
-        <v>411</v>
       </c>
       <c r="E27" s="7">
         <v>4</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="G27" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7182,22 +7188,22 @@
         <v>10</v>
       </c>
       <c r="C28" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D28" s="8" t="s">
         <v>413</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>414</v>
       </c>
       <c r="E28" s="7">
         <v>4</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="G28" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7208,22 +7214,22 @@
         <v>10</v>
       </c>
       <c r="C29" s="7" t="s">
+        <v>414</v>
+      </c>
+      <c r="D29" s="8" t="s">
         <v>415</v>
       </c>
-      <c r="D29" s="8" t="s">
-        <v>416</v>
-      </c>
       <c r="E29" s="7">
         <v>3</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="G29" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7234,22 +7240,22 @@
         <v>21</v>
       </c>
       <c r="C30" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="D30" s="8" t="s">
         <v>417</v>
-      </c>
-      <c r="D30" s="8" t="s">
-        <v>418</v>
       </c>
       <c r="E30" s="7">
         <v>4</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="G30" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7260,22 +7266,22 @@
         <v>21</v>
       </c>
       <c r="C31" s="7" t="s">
+        <v>419</v>
+      </c>
+      <c r="D31" s="8" t="s">
         <v>420</v>
       </c>
-      <c r="D31" s="8" t="s">
-        <v>421</v>
-      </c>
       <c r="E31" s="7">
         <v>3</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="G31" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7286,22 +7292,22 @@
         <v>21</v>
       </c>
       <c r="C32" s="7" t="s">
+        <v>421</v>
+      </c>
+      <c r="D32" s="8" t="s">
         <v>422</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>423</v>
       </c>
       <c r="E32" s="7">
         <v>4</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="G32" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7312,22 +7318,22 @@
         <v>21</v>
       </c>
       <c r="C33" s="7" t="s">
+        <v>423</v>
+      </c>
+      <c r="D33" s="8" t="s">
         <v>424</v>
-      </c>
-      <c r="D33" s="8" t="s">
-        <v>425</v>
       </c>
       <c r="E33" s="7">
         <v>4</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="G33" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7338,22 +7344,22 @@
         <v>21</v>
       </c>
       <c r="C34" s="7" t="s">
+        <v>426</v>
+      </c>
+      <c r="D34" s="8" t="s">
         <v>427</v>
       </c>
-      <c r="D34" s="8" t="s">
-        <v>428</v>
-      </c>
       <c r="E34" s="7">
         <v>3</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="G34" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H34" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7379,7 +7385,7 @@
         <v>13</v>
       </c>
       <c r="H35" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7393,7 +7399,7 @@
         <v>179</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="E36" s="7">
         <v>3</v>
@@ -7405,7 +7411,7 @@
         <v>13</v>
       </c>
       <c r="H36" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7416,22 +7422,22 @@
         <v>10</v>
       </c>
       <c r="C37" s="7" t="s">
+        <v>429</v>
+      </c>
+      <c r="D37" s="8" t="s">
         <v>430</v>
-      </c>
-      <c r="D37" s="8" t="s">
-        <v>431</v>
       </c>
       <c r="E37" s="7">
         <v>4</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="G37" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H37" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7442,22 +7448,22 @@
         <v>10</v>
       </c>
       <c r="C38" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="D38" s="8" t="s">
         <v>432</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>433</v>
       </c>
       <c r="E38" s="7">
         <v>4</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="G38" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H38" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7468,22 +7474,22 @@
         <v>10</v>
       </c>
       <c r="C39" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="D39" s="8" t="s">
         <v>435</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>436</v>
       </c>
       <c r="E39" s="7">
         <v>4</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="G39" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H39" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7497,7 +7503,7 @@
         <v>179</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="E40" s="7">
         <v>3</v>
@@ -7509,7 +7515,7 @@
         <v>13</v>
       </c>
       <c r="H40" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7523,7 +7529,7 @@
         <v>179</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="E41" s="7">
         <v>3</v>
@@ -7535,7 +7541,7 @@
         <v>13</v>
       </c>
       <c r="H41" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7546,22 +7552,22 @@
         <v>21</v>
       </c>
       <c r="C42" s="7" t="s">
+        <v>438</v>
+      </c>
+      <c r="D42" s="8" t="s">
         <v>439</v>
       </c>
-      <c r="D42" s="8" t="s">
-        <v>440</v>
-      </c>
       <c r="E42" s="7">
         <v>3</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="G42" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H42" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7572,22 +7578,22 @@
         <v>21</v>
       </c>
       <c r="C43" s="7" t="s">
+        <v>440</v>
+      </c>
+      <c r="D43" s="8" t="s">
         <v>441</v>
-      </c>
-      <c r="D43" s="8" t="s">
-        <v>442</v>
       </c>
       <c r="E43" s="7">
         <v>4</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="G43" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H43" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7598,7 +7604,7 @@
         <v>21</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="D44" s="8" t="s">
         <v>89</v>
@@ -7607,13 +7613,13 @@
         <v>5</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="G44" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H44" s="8" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -7624,22 +7630,22 @@
         <v>13</v>
       </c>
       <c r="C45" s="7" t="s">
+        <v>444</v>
+      </c>
+      <c r="D45" s="8" t="s">
         <v>445</v>
-      </c>
-      <c r="D45" s="8" t="s">
-        <v>446</v>
       </c>
       <c r="E45" s="7">
         <v>2</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="G45" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H45" s="8" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7650,10 +7656,10 @@
         <v>13</v>
       </c>
       <c r="C46" s="7" t="s">
+        <v>447</v>
+      </c>
+      <c r="D46" s="8" t="s">
         <v>448</v>
-      </c>
-      <c r="D46" s="8" t="s">
-        <v>449</v>
       </c>
       <c r="E46" s="7">
         <v>4</v>
@@ -7665,7 +7671,7 @@
         <v>13</v>
       </c>
       <c r="H46" s="8" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7676,22 +7682,22 @@
         <v>13</v>
       </c>
       <c r="C47" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="D47" s="8" t="s">
         <v>451</v>
-      </c>
-      <c r="D47" s="8" t="s">
-        <v>452</v>
       </c>
       <c r="E47" s="7">
         <v>2</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="G47" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H47" s="8" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7702,22 +7708,22 @@
         <v>13</v>
       </c>
       <c r="C48" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="D48" s="8" t="s">
         <v>453</v>
-      </c>
-      <c r="D48" s="8" t="s">
-        <v>454</v>
       </c>
       <c r="E48" s="7">
         <v>4</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="G48" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H48" s="8" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7728,22 +7734,22 @@
         <v>13</v>
       </c>
       <c r="C49" s="7" t="s">
+        <v>455</v>
+      </c>
+      <c r="D49" s="8" t="s">
         <v>456</v>
-      </c>
-      <c r="D49" s="8" t="s">
-        <v>457</v>
       </c>
       <c r="E49" s="7">
         <v>4</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="G49" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H49" s="8" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7754,72 +7760,72 @@
         <v>13</v>
       </c>
       <c r="C50" s="7" t="s">
+        <v>458</v>
+      </c>
+      <c r="D50" s="8" t="s">
         <v>459</v>
-      </c>
-      <c r="D50" s="8" t="s">
-        <v>460</v>
       </c>
       <c r="E50" s="7">
         <v>4</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="G50" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H50" s="8" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="9" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" s="9" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" s="9" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" s="9" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" s="9" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" s="9" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" s="9" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" s="9" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" s="9" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
   </sheetData>
@@ -7843,12 +7849,12 @@
   <sheetData>
     <row r="1" spans="1:8" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -7885,22 +7891,22 @@
         <v>10</v>
       </c>
       <c r="C5" s="7" t="s">
+        <v>473</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>474</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="E5" s="7">
+        <v>3</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="8" t="s">
         <v>475</v>
-      </c>
-      <c r="E5" s="7">
-        <v>3</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="8" t="s">
-        <v>476</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7926,7 +7932,7 @@
         <v>13</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7937,11 +7943,11 @@
         <v>10</v>
       </c>
       <c r="C7" s="7" t="s">
+        <v>476</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>477</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>478</v>
-      </c>
       <c r="E7" s="7">
         <v>3</v>
       </c>
@@ -7952,7 +7958,7 @@
         <v>13</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -7978,7 +7984,7 @@
         <v>13</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -8004,7 +8010,7 @@
         <v>13</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -8015,22 +8021,22 @@
         <v>21</v>
       </c>
       <c r="C10" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>479</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="E10" s="7">
+        <v>3</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>473</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="8" t="s">
         <v>480</v>
-      </c>
-      <c r="E10" s="7">
-        <v>3</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>474</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>481</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
@@ -8041,10 +8047,10 @@
         <v>21</v>
       </c>
       <c r="C11" s="7" t="s">
+        <v>481</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>482</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>483</v>
       </c>
       <c r="E11" s="7">
         <v>3</v>
@@ -8056,7 +8062,7 @@
         <v>13</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -8082,7 +8088,7 @@
         <v>13</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -8108,7 +8114,7 @@
         <v>13</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -8122,7 +8128,7 @@
         <v>19</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="E14" s="7">
         <v>4</v>
@@ -8134,7 +8140,7 @@
         <v>13</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
@@ -8145,22 +8151,22 @@
         <v>10</v>
       </c>
       <c r="C15" s="7" t="s">
+        <v>484</v>
+      </c>
+      <c r="D15" s="8" t="s">
         <v>485</v>
       </c>
-      <c r="D15" s="8" t="s">
-        <v>486</v>
-      </c>
       <c r="E15" s="7">
         <v>3</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="G15" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
@@ -8171,22 +8177,22 @@
         <v>10</v>
       </c>
       <c r="C16" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>487</v>
       </c>
-      <c r="D16" s="8" t="s">
-        <v>488</v>
-      </c>
       <c r="E16" s="7">
         <v>3</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="G16" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -8197,22 +8203,22 @@
         <v>10</v>
       </c>
       <c r="C17" s="7" t="s">
+        <v>488</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>489</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="E17" s="7">
+        <v>3</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>473</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" s="8" t="s">
         <v>490</v>
-      </c>
-      <c r="E17" s="7">
-        <v>3</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>474</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>491</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -8223,10 +8229,10 @@
         <v>10</v>
       </c>
       <c r="C18" s="7" t="s">
+        <v>491</v>
+      </c>
+      <c r="D18" s="8" t="s">
         <v>492</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>493</v>
       </c>
       <c r="E18" s="7">
         <v>3</v>
@@ -8238,7 +8244,7 @@
         <v>13</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
@@ -8252,19 +8258,19 @@
         <v>29</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="E19" s="7">
         <v>4</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="G19" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
@@ -8275,22 +8281,22 @@
         <v>21</v>
       </c>
       <c r="C20" s="7" t="s">
+        <v>496</v>
+      </c>
+      <c r="D20" s="8" t="s">
         <v>497</v>
       </c>
-      <c r="D20" s="8" t="s">
-        <v>498</v>
-      </c>
       <c r="E20" s="7">
         <v>3</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="G20" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
@@ -8301,22 +8307,22 @@
         <v>21</v>
       </c>
       <c r="C21" s="7" t="s">
+        <v>498</v>
+      </c>
+      <c r="D21" s="8" t="s">
         <v>499</v>
       </c>
-      <c r="D21" s="8" t="s">
-        <v>500</v>
-      </c>
       <c r="E21" s="7">
         <v>3</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="G21" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
@@ -8327,22 +8333,22 @@
         <v>21</v>
       </c>
       <c r="C22" s="7" t="s">
+        <v>500</v>
+      </c>
+      <c r="D22" s="8" t="s">
         <v>501</v>
       </c>
-      <c r="D22" s="8" t="s">
-        <v>502</v>
-      </c>
       <c r="E22" s="7">
         <v>3</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="G22" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
@@ -8353,22 +8359,22 @@
         <v>21</v>
       </c>
       <c r="C23" s="7" t="s">
+        <v>502</v>
+      </c>
+      <c r="D23" s="8" t="s">
         <v>503</v>
       </c>
-      <c r="D23" s="8" t="s">
-        <v>504</v>
-      </c>
       <c r="E23" s="7">
         <v>3</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="G23" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -8379,22 +8385,22 @@
         <v>21</v>
       </c>
       <c r="C24" s="7" t="s">
+        <v>504</v>
+      </c>
+      <c r="D24" s="8" t="s">
         <v>505</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="E24" s="7">
+        <v>3</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>491</v>
+      </c>
+      <c r="G24" s="11" t="s">
         <v>506</v>
       </c>
-      <c r="E24" s="7">
-        <v>3</v>
-      </c>
-      <c r="F24" s="8" t="s">
-        <v>492</v>
-      </c>
-      <c r="G24" s="11" t="s">
+      <c r="H24" s="8" t="s">
         <v>507</v>
-      </c>
-      <c r="H24" s="8" t="s">
-        <v>508</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -8405,22 +8411,22 @@
         <v>21</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="D25" s="8" t="s">
+        <v>508</v>
+      </c>
+      <c r="E25" s="7">
+        <v>3</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>504</v>
+      </c>
+      <c r="H25" s="8" t="s">
         <v>509</v>
-      </c>
-      <c r="E25" s="7">
-        <v>3</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25" s="8" t="s">
-        <v>505</v>
-      </c>
-      <c r="H25" s="8" t="s">
-        <v>510</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
@@ -8431,22 +8437,22 @@
         <v>10</v>
       </c>
       <c r="C26" s="7" t="s">
+        <v>510</v>
+      </c>
+      <c r="D26" s="8" t="s">
         <v>511</v>
       </c>
-      <c r="D26" s="8" t="s">
-        <v>512</v>
-      </c>
       <c r="E26" s="7">
         <v>3</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="G26" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
@@ -8457,22 +8463,22 @@
         <v>10</v>
       </c>
       <c r="C27" s="7" t="s">
+        <v>512</v>
+      </c>
+      <c r="D27" s="8" t="s">
         <v>513</v>
       </c>
-      <c r="D27" s="8" t="s">
-        <v>514</v>
-      </c>
       <c r="E27" s="7">
         <v>3</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="G27" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
@@ -8483,22 +8489,22 @@
         <v>10</v>
       </c>
       <c r="C28" s="7" t="s">
+        <v>514</v>
+      </c>
+      <c r="D28" s="8" t="s">
         <v>515</v>
       </c>
-      <c r="D28" s="8" t="s">
-        <v>516</v>
-      </c>
       <c r="E28" s="7">
         <v>3</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="G28" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
@@ -8509,22 +8515,22 @@
         <v>10</v>
       </c>
       <c r="C29" s="7" t="s">
+        <v>516</v>
+      </c>
+      <c r="D29" s="8" t="s">
         <v>517</v>
       </c>
-      <c r="D29" s="8" t="s">
-        <v>518</v>
-      </c>
       <c r="E29" s="7">
         <v>3</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="G29" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
@@ -8535,22 +8541,22 @@
         <v>10</v>
       </c>
       <c r="C30" s="7" t="s">
+        <v>518</v>
+      </c>
+      <c r="D30" s="8" t="s">
         <v>519</v>
       </c>
-      <c r="D30" s="8" t="s">
-        <v>520</v>
-      </c>
       <c r="E30" s="7">
         <v>3</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="G30" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
@@ -8561,22 +8567,22 @@
         <v>10</v>
       </c>
       <c r="C31" s="7" t="s">
+        <v>520</v>
+      </c>
+      <c r="D31" s="8" t="s">
         <v>521</v>
       </c>
-      <c r="D31" s="8" t="s">
-        <v>522</v>
-      </c>
       <c r="E31" s="7">
         <v>3</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="G31" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
@@ -8587,22 +8593,22 @@
         <v>21</v>
       </c>
       <c r="C32" s="7" t="s">
+        <v>522</v>
+      </c>
+      <c r="D32" s="8" t="s">
         <v>523</v>
       </c>
-      <c r="D32" s="8" t="s">
-        <v>524</v>
-      </c>
       <c r="E32" s="7">
         <v>3</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="G32" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
@@ -8613,22 +8619,22 @@
         <v>21</v>
       </c>
       <c r="C33" s="7" t="s">
+        <v>524</v>
+      </c>
+      <c r="D33" s="8" t="s">
         <v>525</v>
       </c>
-      <c r="D33" s="8" t="s">
+      <c r="E33" s="7">
+        <v>3</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>512</v>
+      </c>
+      <c r="G33" s="8" t="s">
         <v>526</v>
       </c>
-      <c r="E33" s="7">
-        <v>3</v>
-      </c>
-      <c r="F33" s="8" t="s">
-        <v>513</v>
-      </c>
-      <c r="G33" s="8" t="s">
-        <v>527</v>
-      </c>
       <c r="H33" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -8639,22 +8645,22 @@
         <v>21</v>
       </c>
       <c r="C34" s="7" t="s">
+        <v>527</v>
+      </c>
+      <c r="D34" s="8" t="s">
         <v>528</v>
       </c>
-      <c r="D34" s="8" t="s">
+      <c r="E34" s="7">
+        <v>3</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>514</v>
+      </c>
+      <c r="G34" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H34" s="8" t="s">
         <v>529</v>
-      </c>
-      <c r="E34" s="7">
-        <v>3</v>
-      </c>
-      <c r="F34" s="8" t="s">
-        <v>515</v>
-      </c>
-      <c r="G34" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H34" s="8" t="s">
-        <v>530</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
@@ -8665,22 +8671,22 @@
         <v>21</v>
       </c>
       <c r="C35" s="7" t="s">
+        <v>530</v>
+      </c>
+      <c r="D35" s="8" t="s">
         <v>531</v>
       </c>
-      <c r="D35" s="8" t="s">
-        <v>532</v>
-      </c>
       <c r="E35" s="7">
         <v>3</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="G35" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H35" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -8691,22 +8697,22 @@
         <v>21</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="D36" s="8" t="s">
+        <v>532</v>
+      </c>
+      <c r="E36" s="7">
+        <v>3</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>518</v>
+      </c>
+      <c r="G36" s="8" t="s">
+        <v>524</v>
+      </c>
+      <c r="H36" s="8" t="s">
         <v>533</v>
-      </c>
-      <c r="E36" s="7">
-        <v>3</v>
-      </c>
-      <c r="F36" s="8" t="s">
-        <v>519</v>
-      </c>
-      <c r="G36" s="8" t="s">
-        <v>525</v>
-      </c>
-      <c r="H36" s="8" t="s">
-        <v>534</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
@@ -8717,22 +8723,22 @@
         <v>21</v>
       </c>
       <c r="C37" s="7" t="s">
+        <v>534</v>
+      </c>
+      <c r="D37" s="8" t="s">
         <v>535</v>
       </c>
-      <c r="D37" s="8" t="s">
-        <v>536</v>
-      </c>
       <c r="E37" s="7">
         <v>3</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H37" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
@@ -8743,22 +8749,22 @@
         <v>10</v>
       </c>
       <c r="C38" s="7" t="s">
+        <v>536</v>
+      </c>
+      <c r="D38" s="8" t="s">
         <v>537</v>
       </c>
-      <c r="D38" s="8" t="s">
-        <v>538</v>
-      </c>
       <c r="E38" s="7">
         <v>3</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="G38" s="8" t="s">
         <v>13</v>
       </c>
       <c r="H38" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -8769,20 +8775,20 @@
         <v>10</v>
       </c>
       <c r="C39" s="7" t="s">
+        <v>538</v>
+      </c>
+      <c r="D39" s="8" t="s">
         <v>539</v>
       </c>
-      <c r="D39" s="8" t="s">
-        <v>540</v>
-      </c>
       <c r="E39" s="7">
         <v>3</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="G39" s="8"/>
       <c r="H39" s="8" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
@@ -8793,22 +8799,22 @@
         <v>10</v>
       </c>
       <c r="C40" s="7" t="s">
+        <v>541</v>
+      </c>
+      <c r="D40" s="8" t="s">
         <v>542</v>
       </c>
-      <c r="D40" s="8" t="s">
-        <v>543</v>
-      </c>
       <c r="E40" s="7">
         <v>3</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="G40" s="12" t="s">
         <v>13</v>
       </c>
       <c r="H40" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -8819,22 +8825,22 @@
         <v>10</v>
       </c>
       <c r="C41" s="7" t="s">
+        <v>543</v>
+      </c>
+      <c r="D41" s="8" t="s">
         <v>544</v>
       </c>
-      <c r="D41" s="8" t="s">
+      <c r="E41" s="7">
+        <v>3</v>
+      </c>
+      <c r="F41" s="12" t="s">
         <v>545</v>
       </c>
-      <c r="E41" s="7">
-        <v>3</v>
-      </c>
-      <c r="F41" s="12" t="s">
+      <c r="G41" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H41" s="8" t="s">
         <v>546</v>
-      </c>
-      <c r="G41" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H41" s="8" t="s">
-        <v>547</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -8848,7 +8854,7 @@
         <v>13</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="E42" s="7">
         <v>3</v>
@@ -8860,7 +8866,7 @@
         <v>13</v>
       </c>
       <c r="H42" s="8" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -8874,7 +8880,7 @@
         <v>13</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="E43" s="7">
         <v>3</v>
@@ -8886,7 +8892,7 @@
         <v>13</v>
       </c>
       <c r="H43" s="8" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.3">
@@ -8897,22 +8903,22 @@
         <v>21</v>
       </c>
       <c r="C44" s="7" t="s">
+        <v>549</v>
+      </c>
+      <c r="D44" s="8" t="s">
         <v>550</v>
       </c>
-      <c r="D44" s="8" t="s">
+      <c r="E44" s="7">
+        <v>3</v>
+      </c>
+      <c r="F44" s="8" t="s">
         <v>551</v>
       </c>
-      <c r="E44" s="7">
-        <v>3</v>
-      </c>
-      <c r="F44" s="8" t="s">
+      <c r="G44" s="8" t="s">
         <v>552</v>
       </c>
-      <c r="G44" s="8" t="s">
-        <v>553</v>
-      </c>
       <c r="H44" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -8923,22 +8929,22 @@
         <v>21</v>
       </c>
       <c r="C45" s="7" t="s">
+        <v>552</v>
+      </c>
+      <c r="D45" s="8" t="s">
         <v>553</v>
       </c>
-      <c r="D45" s="8" t="s">
+      <c r="E45" s="7">
+        <v>3</v>
+      </c>
+      <c r="F45" s="8" t="s">
+        <v>538</v>
+      </c>
+      <c r="G45" s="11" t="s">
+        <v>549</v>
+      </c>
+      <c r="H45" s="8" t="s">
         <v>554</v>
-      </c>
-      <c r="E45" s="7">
-        <v>3</v>
-      </c>
-      <c r="F45" s="8" t="s">
-        <v>539</v>
-      </c>
-      <c r="G45" s="11" t="s">
-        <v>550</v>
-      </c>
-      <c r="H45" s="8" t="s">
-        <v>555</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -8949,22 +8955,22 @@
         <v>21</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E46" s="7">
         <v>6</v>
       </c>
       <c r="F46" s="8" t="s">
+        <v>556</v>
+      </c>
+      <c r="G46" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H46" s="8" t="s">
         <v>557</v>
-      </c>
-      <c r="G46" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H46" s="8" t="s">
-        <v>558</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
@@ -8978,13 +8984,13 @@
         <v>13</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="E47" s="7">
         <v>3</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="G47" s="8" t="s">
         <v>13</v>
@@ -9002,13 +9008,13 @@
         <v>13</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="E48" s="7">
         <v>3</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="G48" s="8" t="s">
         <v>13</v>
@@ -9017,37 +9023,37 @@
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" s="9" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" s="9" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" s="9" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" s="9" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" s="9" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" s="9" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" s="9" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.3">
@@ -9055,12 +9061,12 @@
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A58" s="9" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" s="9" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
   </sheetData>

</xml_diff>